<commit_message>
coding egg and chicken movements - not yet tested
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89A8852-824E-4EA0-A156-4C536C1CBD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8E9615-8012-41E1-92BB-E727D96CC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
   <sheets>
     <sheet name="PoultryMovement" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="15">
   <si>
     <t>From</t>
   </si>
@@ -460,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D572A8AD-8BDA-4C19-ADD0-7A9D92D57BA2}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.875" customWidth="1"/>
@@ -660,6 +660,20 @@
         <v>7</v>
       </c>
       <c r="D14">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15">
         <v>546</v>
       </c>
     </row>

</xml_diff>

<commit_message>
renaming meat growing-farm to broiler farm
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8E9615-8012-41E1-92BB-E727D96CC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6840BA85-F131-4C7E-AD1D-B4DD22FC2B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
+    <workbookView xWindow="6300" yWindow="1875" windowWidth="21600" windowHeight="11295" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
   <sheets>
     <sheet name="PoultryMovement" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="16">
   <si>
     <t>From</t>
   </si>
@@ -54,9 +54,6 @@
     <t>hatchery</t>
   </si>
   <si>
-    <t>pullets farm</t>
-  </si>
-  <si>
     <t>meat growing-farm</t>
   </si>
   <si>
@@ -82,6 +79,12 @@
   </si>
   <si>
     <t>egg processing</t>
+  </si>
+  <si>
+    <t>pullet farm</t>
+  </si>
+  <si>
+    <t>broiler farm</t>
   </si>
 </sst>
 </file>
@@ -486,10 +489,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -500,10 +503,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -511,13 +514,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4">
         <v>119</v>
@@ -525,13 +528,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5">
         <v>119</v>
@@ -539,13 +542,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6">
         <v>119</v>
@@ -553,13 +556,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7">
         <v>119</v>
@@ -567,13 +570,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
         <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -581,13 +584,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -595,13 +598,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -609,13 +612,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D11">
         <v>50</v>
@@ -623,13 +626,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D12">
         <v>546</v>
@@ -637,13 +640,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13">
         <v>546</v>
@@ -651,13 +654,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
       <c r="C14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D14">
         <v>546</v>
@@ -668,10 +671,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D15">
         <v>546</v>
@@ -692,7 +695,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
putting a capacity limit on properties
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6840BA85-F131-4C7E-AD1D-B4DD22FC2B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89074A15-359E-4176-84E0-A54712D23A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6300" yWindow="1875" windowWidth="21600" windowHeight="11295" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="15">
   <si>
     <t>From</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>hatchery</t>
-  </si>
-  <si>
-    <t>meat growing-farm</t>
   </si>
   <si>
     <t>chicken</t>
@@ -489,10 +486,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -503,10 +500,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -514,13 +511,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>119</v>
@@ -528,13 +525,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>119</v>
@@ -542,13 +539,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>119</v>
@@ -556,13 +553,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>119</v>
@@ -570,13 +567,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
         <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -584,13 +581,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -598,13 +595,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -612,13 +609,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>50</v>
@@ -626,13 +623,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>546</v>
@@ -640,13 +637,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>546</v>
@@ -654,13 +651,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
         <v>11</v>
       </c>
-      <c r="B14" t="s">
-        <v>12</v>
-      </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>546</v>
@@ -671,10 +668,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15">
         <v>546</v>
@@ -695,7 +692,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added possible movements from hatcheries to layers
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89074A15-359E-4176-84E0-A54712D23A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20661A10-5130-4D27-B149-FEA6981EFA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6300" yWindow="1875" windowWidth="21600" windowHeight="11295" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
   <sheets>
     <sheet name="PoultryMovement" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="17">
   <si>
     <t>From</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>broiler farm</t>
+  </si>
+  <si>
+    <t>Freeform notes</t>
+  </si>
+  <si>
+    <t>only sufficiently large farms will accept hatchlings (inside code)</t>
   </si>
 </sst>
 </file>
@@ -460,14 +466,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D572A8AD-8BDA-4C19-ADD0-7A9D92D57BA2}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.875" customWidth="1"/>
     <col min="2" max="2" width="19.875" customWidth="1"/>
+    <col min="5" max="5" width="52.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -480,8 +487,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -495,7 +505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -508,10 +518,13 @@
       <c r="D3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -520,12 +533,15 @@
         <v>5</v>
       </c>
       <c r="D4">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -534,12 +550,15 @@
         <v>5</v>
       </c>
       <c r="D5">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -548,15 +567,18 @@
         <v>5</v>
       </c>
       <c r="D6">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -565,93 +587,93 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C11" t="s">
         <v>8</v>
       </c>
-      <c r="D8">
+      <c r="D11">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C12" t="s">
         <v>8</v>
       </c>
-      <c r="D9">
+      <c r="D12">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B13" t="s">
         <v>12</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C13" t="s">
         <v>8</v>
       </c>
-      <c r="D10">
+      <c r="D13">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>10</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
@@ -660,12 +682,12 @@
         <v>5</v>
       </c>
       <c r="D14">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
@@ -674,6 +696,48 @@
         <v>5</v>
       </c>
       <c r="D15">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18">
         <v>546</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removed movement from pullet farm to broiler
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20661A10-5130-4D27-B149-FEA6981EFA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55745367-862C-4518-BA79-ECEA48B736E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="17">
   <si>
     <t>From</t>
   </si>
@@ -466,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D572A8AD-8BDA-4C19-ADD0-7A9D92D57BA2}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.875" customWidth="1"/>
@@ -617,21 +617,21 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
@@ -645,7 +645,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
@@ -659,21 +659,21 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
@@ -682,12 +682,12 @@
         <v>5</v>
       </c>
       <c r="D14">
-        <v>50</v>
+        <v>546</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
@@ -701,7 +701,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
@@ -715,7 +715,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
@@ -724,20 +724,6 @@
         <v>5</v>
       </c>
       <c r="D17">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18">
         <v>546</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added in breeder farms and refactored the initial init for chickens and eggs, and chicken/egg dicts
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55745367-862C-4518-BA79-ECEA48B736E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE4BF376-B8BC-40FA-A35F-831CC65C5A43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
+    <workbookView xWindow="38865" yWindow="255" windowWidth="18645" windowHeight="14895" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
   <sheets>
     <sheet name="PoultryMovement" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="18">
   <si>
     <t>From</t>
   </si>
@@ -88,6 +88,9 @@
   </si>
   <si>
     <t>only sufficiently large farms will accept hatchlings (inside code)</t>
+  </si>
+  <si>
+    <t>breeder</t>
   </si>
 </sst>
 </file>
@@ -466,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D572A8AD-8BDA-4C19-ADD0-7A9D92D57BA2}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.875" customWidth="1"/>
@@ -715,7 +718,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
@@ -725,6 +728,34 @@
       </c>
       <c r="D17">
         <v>546</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactoring movement code (incomplete)
</commit_message>
<xml_diff>
--- a/data/MovementNetwork.xlsx
+++ b/data/MovementNetwork.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE4BF376-B8BC-40FA-A35F-831CC65C5A43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA98DDC6-FB8D-4EBC-9BAD-F115681976C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38865" yWindow="255" windowWidth="18645" windowHeight="14895" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
+    <workbookView xWindow="30675" yWindow="375" windowWidth="23640" windowHeight="14895" xr2:uid="{AA6F4960-0E47-4544-988D-5FCF85614375}"/>
   </bookViews>
   <sheets>
     <sheet name="PoultryMovement" sheetId="1" r:id="rId1"/>

</xml_diff>